<commit_message>
Add contractual availability to August monthly report
Add a Contractual Availability card to the Overview and a per-turbine
monthly contractual availability block to Turbine & PCS Detail, in both
the site page and the downloadable xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/reports/monthly/Dassiesridge-Monthly-KPI-Matrix-2026-08.xlsx
+++ b/public/reports/monthly/Dassiesridge-Monthly-KPI-Matrix-2026-08.xlsx
@@ -286,12 +286,12 @@
     <author>ReportHub</author>
   </authors>
   <commentList>
-    <comment ref="A42" authorId="0" shapeId="0">
+    <comment ref="A61" authorId="0" shapeId="0">
       <text>
         <t>Lost energy = MWh the turbine failed to produce due to unavailability (outages, curtailment for cause). A turbine can rank mid-table on availability % but still top this list if its outages happened during high-wind periods -- % alone doesn't capture that.</t>
       </text>
     </comment>
-    <comment ref="A60" authorId="0" shapeId="0">
+    <comment ref="A79" authorId="0" shapeId="0">
       <text>
         <t>PCS (Battery Inverter) monitoring data is only available from 1 July 2026 onward -- Jan-Jun cells are marked n/a rather than estimated. PCS11 is the fleet's weakest unit in both months of available data (84.1% Jul, 77.9% Aug).</t>
       </text>
@@ -2654,7 +2654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3902,7 +3902,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>TURBINE MONTHLY LOST ENERGY (MWh, unavailability)</t>
+          <t>TURBINE MONTHLY CONTRACTUAL AVAILABILITY (%)</t>
         </is>
       </c>
       <c r="B42" s="3" t="n"/>
@@ -3975,32 +3975,32 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C44" s="10" t="n">
-        <v>90.341156</v>
+        <v>99.62777786526684</v>
       </c>
       <c r="D44" s="10" t="n">
-        <v>123.918777</v>
+        <v>96.1730046444122</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>55.514584</v>
+        <v>94.98932840068298</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>100.565176</v>
+        <v>96.12295372656607</v>
       </c>
       <c r="G44" s="10" t="n">
-        <v>171.554548</v>
+        <v>83.22978904584221</v>
       </c>
       <c r="H44" s="10" t="n">
-        <v>472.044306</v>
+        <v>69.41391941391942</v>
       </c>
       <c r="I44" s="10" t="n">
-        <v>44.900924</v>
+        <v>100</v>
       </c>
       <c r="J44" s="10" t="n">
-        <v>65.659099</v>
+        <v>99.16284987277353</v>
       </c>
     </row>
     <row r="45">
@@ -4011,32 +4011,32 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C45" s="10" t="n">
-        <v>80.993386</v>
+        <v>99.41644431089743</v>
       </c>
       <c r="D45" s="10" t="n">
-        <v>86.225369</v>
+        <v>99.03414755807027</v>
       </c>
       <c r="E45" s="10" t="n">
-        <v>27.811788</v>
+        <v>99.97017748036077</v>
       </c>
       <c r="F45" s="10" t="n">
-        <v>82.116669</v>
+        <v>96.11585251731238</v>
       </c>
       <c r="G45" s="10" t="n">
-        <v>160.941136</v>
+        <v>93.99462997562956</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>544.558187</v>
+        <v>62.86471642826181</v>
       </c>
       <c r="I45" s="10" t="n">
-        <v>66.316266</v>
+        <v>96.98302055406613</v>
       </c>
       <c r="J45" s="10" t="n">
-        <v>79.837789</v>
+        <v>99.46841327573394</v>
       </c>
     </row>
     <row r="46">
@@ -4047,32 +4047,32 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C46" s="10" t="n">
-        <v>74.01553800000001</v>
+        <v>99.59667451706802</v>
       </c>
       <c r="D46" s="10" t="n">
-        <v>84.74361</v>
+        <v>99.80472967479675</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>35.218166</v>
+        <v>99.74157577062989</v>
       </c>
       <c r="F46" s="10" t="n">
-        <v>36.893027</v>
+        <v>98.54128519136317</v>
       </c>
       <c r="G46" s="10" t="n">
-        <v>167.78334</v>
+        <v>95.88156123822343</v>
       </c>
       <c r="H46" s="10" t="n">
-        <v>511.023418</v>
+        <v>68.8794476898566</v>
       </c>
       <c r="I46" s="10" t="n">
-        <v>48.131542</v>
+        <v>99.91336505808758</v>
       </c>
       <c r="J46" s="10" t="n">
-        <v>59.22373</v>
+        <v>99.82693180786345</v>
       </c>
     </row>
     <row r="47">
@@ -4083,32 +4083,32 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C47" s="10" t="n">
-        <v>118.783906</v>
+        <v>97.32098107171421</v>
       </c>
       <c r="D47" s="10" t="n">
-        <v>118.207259</v>
+        <v>94.81861378631217</v>
       </c>
       <c r="E47" s="10" t="n">
-        <v>83.65647300000001</v>
+        <v>89.57850276725895</v>
       </c>
       <c r="F47" s="10" t="n">
-        <v>42.321359</v>
+        <v>98.93005340622372</v>
       </c>
       <c r="G47" s="10" t="n">
-        <v>207.141052</v>
+        <v>91.06623172057625</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>448.252119</v>
+        <v>64.80993798650752</v>
       </c>
       <c r="I47" s="10" t="n">
-        <v>60.76895</v>
+        <v>97.40294583979329</v>
       </c>
       <c r="J47" s="10" t="n">
-        <v>124.463486</v>
+        <v>96.0914768184342</v>
       </c>
     </row>
     <row r="48">
@@ -4119,32 +4119,32 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C48" s="10" t="n">
-        <v>108.401945</v>
+        <v>96.96851394440003</v>
       </c>
       <c r="D48" s="10" t="n">
-        <v>119.145319</v>
+        <v>97.04055223806695</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>48.406552</v>
+        <v>98.98955616517469</v>
       </c>
       <c r="F48" s="10" t="n">
-        <v>70.544394</v>
+        <v>99.85950018590816</v>
       </c>
       <c r="G48" s="10" t="n">
-        <v>153.550084</v>
+        <v>95.91673423059667</v>
       </c>
       <c r="H48" s="10" t="n">
-        <v>426.901381</v>
+        <v>68.69846956829441</v>
       </c>
       <c r="I48" s="10" t="n">
-        <v>42.689851</v>
+        <v>99.7548959294576</v>
       </c>
       <c r="J48" s="10" t="n">
-        <v>65.125101</v>
+        <v>97.57679648930335</v>
       </c>
     </row>
     <row r="49">
@@ -4155,32 +4155,32 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C49" s="10" t="n">
-        <v>112.329665</v>
+        <v>98.84295050291159</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>125.84266</v>
+        <v>98.37435753079235</v>
       </c>
       <c r="E49" s="10" t="n">
-        <v>34.564937</v>
+        <v>99.95792027958818</v>
       </c>
       <c r="F49" s="10" t="n">
-        <v>15.420853</v>
+        <v>100</v>
       </c>
       <c r="G49" s="10" t="n">
-        <v>149.382085</v>
+        <v>95.90055351722907</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>510.114279</v>
+        <v>66.44800544830545</v>
       </c>
       <c r="I49" s="10" t="n">
-        <v>39.0727</v>
+        <v>99.16885120643431</v>
       </c>
       <c r="J49" s="10" t="n">
-        <v>33.857889</v>
+        <v>99.8065712329977</v>
       </c>
     </row>
     <row r="50">
@@ -4191,32 +4191,32 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C50" s="10" t="n">
-        <v>82.395867</v>
+        <v>99.20145973416732</v>
       </c>
       <c r="D50" s="10" t="n">
-        <v>85.405315</v>
+        <v>99.97721972352025</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>39.474884</v>
+        <v>99.96845972686734</v>
       </c>
       <c r="F50" s="10" t="n">
-        <v>42.371912</v>
+        <v>98.36973579339143</v>
       </c>
       <c r="G50" s="10" t="n">
-        <v>190.628941</v>
+        <v>95.44341459216102</v>
       </c>
       <c r="H50" s="10" t="n">
-        <v>485.492332</v>
+        <v>69.30565704960836</v>
       </c>
       <c r="I50" s="10" t="n">
-        <v>50.021922</v>
+        <v>100</v>
       </c>
       <c r="J50" s="10" t="n">
-        <v>59.099455</v>
+        <v>99.81939197697429</v>
       </c>
     </row>
     <row r="51">
@@ -4227,32 +4227,32 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C51" s="10" t="n">
-        <v>103.456171</v>
+        <v>98.69884157754009</v>
       </c>
       <c r="D51" s="10" t="n">
-        <v>100.172993</v>
+        <v>98.99940631808279</v>
       </c>
       <c r="E51" s="10" t="n">
-        <v>27.117473</v>
+        <v>99.98839907192576</v>
       </c>
       <c r="F51" s="10" t="n">
-        <v>43.265019</v>
+        <v>99.98389087301587</v>
       </c>
       <c r="G51" s="10" t="n">
-        <v>143.316595</v>
+        <v>94.4159946191669</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>532.9996169999999</v>
+        <v>63.15629862918619</v>
       </c>
       <c r="I51" s="10" t="n">
-        <v>71.36399900000001</v>
+        <v>97.47887111379414</v>
       </c>
       <c r="J51" s="10" t="n">
-        <v>62.290298</v>
+        <v>97.12800591934887</v>
       </c>
     </row>
     <row r="52">
@@ -4263,32 +4263,32 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C52" s="10" t="n">
-        <v>122.179099</v>
+        <v>98.73328151224153</v>
       </c>
       <c r="D52" s="10" t="n">
-        <v>121.386776</v>
+        <v>98.88544360293417</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>44.494946</v>
+        <v>97.60631978506477</v>
       </c>
       <c r="F52" s="10" t="n">
-        <v>82.84994</v>
+        <v>97.06444279206859</v>
       </c>
       <c r="G52" s="10" t="n">
-        <v>143.238463</v>
+        <v>96.04989604989605</v>
       </c>
       <c r="H52" s="10" t="n">
-        <v>497.97957</v>
+        <v>64.15435849772382</v>
       </c>
       <c r="I52" s="10" t="n">
-        <v>42.738838</v>
+        <v>100</v>
       </c>
       <c r="J52" s="10" t="n">
-        <v>39.809798</v>
+        <v>99.83194790854768</v>
       </c>
     </row>
     <row r="53">
@@ -4299,32 +4299,32 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C53" s="10" t="n">
-        <v>82.920506</v>
+        <v>99.83014933227204</v>
       </c>
       <c r="D53" s="10" t="n">
-        <v>100.485173</v>
+        <v>98.85284105798377</v>
       </c>
       <c r="E53" s="10" t="n">
-        <v>75.55337299999999</v>
+        <v>95.67583860849729</v>
       </c>
       <c r="F53" s="10" t="n">
-        <v>34.882023</v>
+        <v>99.88386242576095</v>
       </c>
       <c r="G53" s="10" t="n">
-        <v>151.497191</v>
+        <v>95.91397849462365</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>431.959576</v>
+        <v>66.60376706410921</v>
       </c>
       <c r="I53" s="10" t="n">
-        <v>48.930094</v>
+        <v>99.99693439607603</v>
       </c>
       <c r="J53" s="10" t="n">
-        <v>100.31041</v>
+        <v>94.45888817876892</v>
       </c>
     </row>
     <row r="54">
@@ -4335,32 +4335,32 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C54" s="10" t="n">
-        <v>149.718974</v>
+        <v>99.20014631357482</v>
       </c>
       <c r="D54" s="10" t="n">
-        <v>78.94345199999999</v>
+        <v>99.66008679927667</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>28.087224</v>
+        <v>99.97231346479435</v>
       </c>
       <c r="F54" s="10" t="n">
-        <v>35.962257</v>
+        <v>98.42541010365203</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>133.372945</v>
+        <v>84.45944336977853</v>
       </c>
       <c r="H54" s="10" t="n">
-        <v>524.589872</v>
+        <v>60.84077328431372</v>
       </c>
       <c r="I54" s="10" t="n">
-        <v>43.022519</v>
+        <v>99.92527173913044</v>
       </c>
       <c r="J54" s="10" t="n">
-        <v>56.678719</v>
+        <v>99.68443784822286</v>
       </c>
     </row>
     <row r="55">
@@ -4371,32 +4371,32 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C55" s="10" t="n">
-        <v>216.974047</v>
+        <v>93.83042902358655</v>
       </c>
       <c r="D55" s="10" t="n">
-        <v>146.532089</v>
+        <v>98.98196015449301</v>
       </c>
       <c r="E55" s="10" t="n">
-        <v>31.842171</v>
+        <v>99.97902612359552</v>
       </c>
       <c r="F55" s="10" t="n">
-        <v>40.789063</v>
+        <v>99.95614512471656</v>
       </c>
       <c r="G55" s="10" t="n">
-        <v>165.086863</v>
+        <v>94.60099190122145</v>
       </c>
       <c r="H55" s="10" t="n">
-        <v>487.499399</v>
+        <v>69.41865594187857</v>
       </c>
       <c r="I55" s="10" t="n">
-        <v>47.575897</v>
+        <v>99.9699732986312</v>
       </c>
       <c r="J55" s="10" t="n">
-        <v>64.345932</v>
+        <v>99.15638192760262</v>
       </c>
     </row>
     <row r="56">
@@ -4407,32 +4407,32 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C56" s="10" t="n">
-        <v>182.324618</v>
+        <v>98.8361365901406</v>
       </c>
       <c r="D56" s="10" t="n">
-        <v>107.578467</v>
+        <v>99.33670227835563</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>35.045967</v>
+        <v>99.92468710876369</v>
       </c>
       <c r="F56" s="10" t="n">
-        <v>52.340176</v>
+        <v>99.52399737015122</v>
       </c>
       <c r="G56" s="10" t="n">
-        <v>162.705752</v>
+        <v>94.54695663845663</v>
       </c>
       <c r="H56" s="10" t="n">
-        <v>507.816809</v>
+        <v>68.15547556625646</v>
       </c>
       <c r="I56" s="10" t="n">
-        <v>44.071363</v>
+        <v>99.97552626200695</v>
       </c>
       <c r="J56" s="10" t="n">
-        <v>81.18752600000001</v>
+        <v>98.56837862114372</v>
       </c>
     </row>
     <row r="57">
@@ -4443,819 +4443,1427 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C57" s="10" t="n">
-        <v>188.823573</v>
+        <v>96.82752992383024</v>
       </c>
       <c r="D57" s="10" t="n">
-        <v>92.174916</v>
+        <v>99.67284377824646</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>48.840233</v>
+        <v>97.19464134709931</v>
       </c>
       <c r="F57" s="10" t="n">
-        <v>31.824552</v>
+        <v>98.34886740041929</v>
       </c>
       <c r="G57" s="10" t="n">
-        <v>229.328235</v>
+        <v>89.43939905781193</v>
       </c>
       <c r="H57" s="10" t="n">
-        <v>423.609727</v>
+        <v>68.80237902135711</v>
       </c>
       <c r="I57" s="10" t="n">
-        <v>65.351546</v>
+        <v>97.61742881097561</v>
       </c>
       <c r="J57" s="10" t="n">
-        <v>53.301366</v>
-      </c>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>PCS (INVERTER) MONTHLY AVAILABILITY (%)</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="n"/>
-      <c r="C60" s="3" t="n"/>
-      <c r="D60" s="3" t="n"/>
-      <c r="E60" s="3" t="n"/>
-      <c r="F60" s="3" t="n"/>
-      <c r="G60" s="3" t="n"/>
-      <c r="H60" s="3" t="n"/>
-      <c r="I60" s="3" t="n"/>
-      <c r="J60" s="3" t="n"/>
-    </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="4" t="inlineStr">
+        <v>98.98995022071945</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Fleet avg</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C58" s="10" t="n">
+        <v>98.34999999999999</v>
+      </c>
+      <c r="D58" s="10" t="n">
+        <v>98.54000000000001</v>
+      </c>
+      <c r="E58" s="10" t="n">
+        <v>98.11</v>
+      </c>
+      <c r="F58" s="10" t="n">
+        <v>98.65000000000001</v>
+      </c>
+      <c r="G58" s="10" t="n">
+        <v>92.95</v>
+      </c>
+      <c r="H58" s="10" t="n">
+        <v>66.52</v>
+      </c>
+      <c r="I58" s="10" t="n">
+        <v>99.16</v>
+      </c>
+      <c r="J58" s="10" t="n">
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>TURBINE MONTHLY LOST ENERGY (MWh, unavailability)</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="n"/>
+      <c r="C61" s="3" t="n"/>
+      <c r="D61" s="3" t="n"/>
+      <c r="E61" s="3" t="n"/>
+      <c r="F61" s="3" t="n"/>
+      <c r="G61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
+      <c r="I61" s="3" t="n"/>
+      <c r="J61" s="3" t="n"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr">
+      <c r="F62" s="5" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="G61" s="5" t="inlineStr">
+      <c r="G62" s="5" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="H61" s="5" t="inlineStr">
+      <c r="H62" s="5" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="I61" s="5" t="inlineStr">
+      <c r="I62" s="5" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="J61" s="5" t="inlineStr">
+      <c r="J62" s="5" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>PCS01</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C62" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D62" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E62" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F62" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G62" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H62" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I62" s="10" t="n">
-        <v>93.51000000000001</v>
-      </c>
-      <c r="J62" s="10" t="n">
-        <v>90.29000000000001</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>PCS02</t>
+          <t>WTG01</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C63" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D63" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E63" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F63" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G63" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H63" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="n">
+        <v>90.341156</v>
+      </c>
+      <c r="D63" s="10" t="n">
+        <v>123.918777</v>
+      </c>
+      <c r="E63" s="10" t="n">
+        <v>55.514584</v>
+      </c>
+      <c r="F63" s="10" t="n">
+        <v>100.565176</v>
+      </c>
+      <c r="G63" s="10" t="n">
+        <v>171.554548</v>
+      </c>
+      <c r="H63" s="10" t="n">
+        <v>472.044306</v>
       </c>
       <c r="I63" s="10" t="n">
-        <v>93.3</v>
+        <v>44.900924</v>
       </c>
       <c r="J63" s="10" t="n">
-        <v>86.95</v>
+        <v>65.659099</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>PCS03</t>
+          <t>WTG16</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C64" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D64" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E64" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F64" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G64" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H64" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="n">
+        <v>80.993386</v>
+      </c>
+      <c r="D64" s="10" t="n">
+        <v>86.225369</v>
+      </c>
+      <c r="E64" s="10" t="n">
+        <v>27.811788</v>
+      </c>
+      <c r="F64" s="10" t="n">
+        <v>82.116669</v>
+      </c>
+      <c r="G64" s="10" t="n">
+        <v>160.941136</v>
+      </c>
+      <c r="H64" s="10" t="n">
+        <v>544.558187</v>
       </c>
       <c r="I64" s="10" t="n">
-        <v>87.15000000000001</v>
+        <v>66.316266</v>
       </c>
       <c r="J64" s="10" t="n">
-        <v>86.14</v>
+        <v>79.837789</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>PCS04</t>
+          <t>WTG20</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C65" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D65" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E65" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F65" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G65" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H65" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="n">
+        <v>74.01553800000001</v>
+      </c>
+      <c r="D65" s="10" t="n">
+        <v>84.74361</v>
+      </c>
+      <c r="E65" s="10" t="n">
+        <v>35.218166</v>
+      </c>
+      <c r="F65" s="10" t="n">
+        <v>36.893027</v>
+      </c>
+      <c r="G65" s="10" t="n">
+        <v>167.78334</v>
+      </c>
+      <c r="H65" s="10" t="n">
+        <v>511.023418</v>
       </c>
       <c r="I65" s="10" t="n">
-        <v>92.36</v>
+        <v>48.131542</v>
       </c>
       <c r="J65" s="10" t="n">
-        <v>90.29000000000001</v>
+        <v>59.22373</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>PCS05</t>
+          <t>WTG21</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C66" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D66" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E66" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F66" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G66" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H66" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C66" s="10" t="n">
+        <v>118.783906</v>
+      </c>
+      <c r="D66" s="10" t="n">
+        <v>118.207259</v>
+      </c>
+      <c r="E66" s="10" t="n">
+        <v>83.65647300000001</v>
+      </c>
+      <c r="F66" s="10" t="n">
+        <v>42.321359</v>
+      </c>
+      <c r="G66" s="10" t="n">
+        <v>207.141052</v>
+      </c>
+      <c r="H66" s="10" t="n">
+        <v>448.252119</v>
       </c>
       <c r="I66" s="10" t="n">
-        <v>86.62</v>
+        <v>60.76895</v>
       </c>
       <c r="J66" s="10" t="n">
-        <v>90.25</v>
+        <v>124.463486</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>PCS06</t>
+          <t>WTG25</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C67" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D67" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E67" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F67" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G67" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H67" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="n">
+        <v>108.401945</v>
+      </c>
+      <c r="D67" s="10" t="n">
+        <v>119.145319</v>
+      </c>
+      <c r="E67" s="10" t="n">
+        <v>48.406552</v>
+      </c>
+      <c r="F67" s="10" t="n">
+        <v>70.544394</v>
+      </c>
+      <c r="G67" s="10" t="n">
+        <v>153.550084</v>
+      </c>
+      <c r="H67" s="10" t="n">
+        <v>426.901381</v>
       </c>
       <c r="I67" s="10" t="n">
-        <v>93.43000000000001</v>
+        <v>42.689851</v>
       </c>
       <c r="J67" s="10" t="n">
-        <v>90.26000000000001</v>
+        <v>65.125101</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>PCS07</t>
+          <t>WTG30</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C68" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D68" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E68" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F68" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G68" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H68" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C68" s="10" t="n">
+        <v>112.329665</v>
+      </c>
+      <c r="D68" s="10" t="n">
+        <v>125.84266</v>
+      </c>
+      <c r="E68" s="10" t="n">
+        <v>34.564937</v>
+      </c>
+      <c r="F68" s="10" t="n">
+        <v>15.420853</v>
+      </c>
+      <c r="G68" s="10" t="n">
+        <v>149.382085</v>
+      </c>
+      <c r="H68" s="10" t="n">
+        <v>510.114279</v>
       </c>
       <c r="I68" s="10" t="n">
-        <v>92.06999999999999</v>
+        <v>39.0727</v>
       </c>
       <c r="J68" s="10" t="n">
-        <v>87.55</v>
+        <v>33.857889</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PCS08</t>
+          <t>WTG52</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C69" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D69" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E69" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F69" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G69" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H69" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C69" s="10" t="n">
+        <v>82.395867</v>
+      </c>
+      <c r="D69" s="10" t="n">
+        <v>85.405315</v>
+      </c>
+      <c r="E69" s="10" t="n">
+        <v>39.474884</v>
+      </c>
+      <c r="F69" s="10" t="n">
+        <v>42.371912</v>
+      </c>
+      <c r="G69" s="10" t="n">
+        <v>190.628941</v>
+      </c>
+      <c r="H69" s="10" t="n">
+        <v>485.492332</v>
       </c>
       <c r="I69" s="10" t="n">
-        <v>92.64</v>
+        <v>50.021922</v>
       </c>
       <c r="J69" s="10" t="n">
-        <v>89.79000000000001</v>
+        <v>59.099455</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PCS09</t>
+          <t>WTG54</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C70" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D70" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E70" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F70" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G70" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H70" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C70" s="10" t="n">
+        <v>103.456171</v>
+      </c>
+      <c r="D70" s="10" t="n">
+        <v>100.172993</v>
+      </c>
+      <c r="E70" s="10" t="n">
+        <v>27.117473</v>
+      </c>
+      <c r="F70" s="10" t="n">
+        <v>43.265019</v>
+      </c>
+      <c r="G70" s="10" t="n">
+        <v>143.316595</v>
+      </c>
+      <c r="H70" s="10" t="n">
+        <v>532.9996169999999</v>
       </c>
       <c r="I70" s="10" t="n">
-        <v>91.95999999999999</v>
+        <v>71.36399900000001</v>
       </c>
       <c r="J70" s="10" t="n">
-        <v>87.19</v>
+        <v>62.290298</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PCS10</t>
+          <t>WTG60</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C71" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D71" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E71" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F71" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G71" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H71" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C71" s="10" t="n">
+        <v>122.179099</v>
+      </c>
+      <c r="D71" s="10" t="n">
+        <v>121.386776</v>
+      </c>
+      <c r="E71" s="10" t="n">
+        <v>44.494946</v>
+      </c>
+      <c r="F71" s="10" t="n">
+        <v>82.84994</v>
+      </c>
+      <c r="G71" s="10" t="n">
+        <v>143.238463</v>
+      </c>
+      <c r="H71" s="10" t="n">
+        <v>497.97957</v>
       </c>
       <c r="I71" s="10" t="n">
-        <v>93.33</v>
+        <v>42.738838</v>
       </c>
       <c r="J71" s="10" t="n">
-        <v>90.25</v>
+        <v>39.809798</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PCS11</t>
+          <t>WTG61</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C72" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D72" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E72" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F72" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G72" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H72" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C72" s="10" t="n">
+        <v>82.920506</v>
+      </c>
+      <c r="D72" s="10" t="n">
+        <v>100.485173</v>
+      </c>
+      <c r="E72" s="10" t="n">
+        <v>75.55337299999999</v>
+      </c>
+      <c r="F72" s="10" t="n">
+        <v>34.882023</v>
+      </c>
+      <c r="G72" s="10" t="n">
+        <v>151.497191</v>
+      </c>
+      <c r="H72" s="10" t="n">
+        <v>431.959576</v>
       </c>
       <c r="I72" s="10" t="n">
-        <v>84.14</v>
+        <v>48.930094</v>
       </c>
       <c r="J72" s="10" t="n">
-        <v>77.87</v>
+        <v>100.31041</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PCS12</t>
+          <t>WTG63</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C73" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D73" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E73" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F73" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G73" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H73" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="n">
+        <v>149.718974</v>
+      </c>
+      <c r="D73" s="10" t="n">
+        <v>78.94345199999999</v>
+      </c>
+      <c r="E73" s="10" t="n">
+        <v>28.087224</v>
+      </c>
+      <c r="F73" s="10" t="n">
+        <v>35.962257</v>
+      </c>
+      <c r="G73" s="10" t="n">
+        <v>133.372945</v>
+      </c>
+      <c r="H73" s="10" t="n">
+        <v>524.589872</v>
       </c>
       <c r="I73" s="10" t="n">
-        <v>93.19</v>
+        <v>43.022519</v>
       </c>
       <c r="J73" s="10" t="n">
-        <v>90.25</v>
+        <v>56.678719</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PCS13</t>
+          <t>WTG64</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C74" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D74" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E74" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F74" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G74" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H74" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="n">
+        <v>216.974047</v>
+      </c>
+      <c r="D74" s="10" t="n">
+        <v>146.532089</v>
+      </c>
+      <c r="E74" s="10" t="n">
+        <v>31.842171</v>
+      </c>
+      <c r="F74" s="10" t="n">
+        <v>40.789063</v>
+      </c>
+      <c r="G74" s="10" t="n">
+        <v>165.086863</v>
+      </c>
+      <c r="H74" s="10" t="n">
+        <v>487.499399</v>
       </c>
       <c r="I74" s="10" t="n">
-        <v>93.17</v>
+        <v>47.575897</v>
       </c>
       <c r="J74" s="10" t="n">
-        <v>90.25</v>
+        <v>64.345932</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PCS14</t>
+          <t>WTG65</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C75" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D75" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E75" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F75" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G75" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H75" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="n">
+        <v>182.324618</v>
+      </c>
+      <c r="D75" s="10" t="n">
+        <v>107.578467</v>
+      </c>
+      <c r="E75" s="10" t="n">
+        <v>35.045967</v>
+      </c>
+      <c r="F75" s="10" t="n">
+        <v>52.340176</v>
+      </c>
+      <c r="G75" s="10" t="n">
+        <v>162.705752</v>
+      </c>
+      <c r="H75" s="10" t="n">
+        <v>507.816809</v>
       </c>
       <c r="I75" s="10" t="n">
-        <v>93.27</v>
+        <v>44.071363</v>
       </c>
       <c r="J75" s="10" t="n">
-        <v>87.65000000000001</v>
+        <v>81.18752600000001</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
+          <t>WTG67</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="n">
+        <v>188.823573</v>
+      </c>
+      <c r="D76" s="10" t="n">
+        <v>92.174916</v>
+      </c>
+      <c r="E76" s="10" t="n">
+        <v>48.840233</v>
+      </c>
+      <c r="F76" s="10" t="n">
+        <v>31.824552</v>
+      </c>
+      <c r="G76" s="10" t="n">
+        <v>229.328235</v>
+      </c>
+      <c r="H76" s="10" t="n">
+        <v>423.609727</v>
+      </c>
+      <c r="I76" s="10" t="n">
+        <v>65.351546</v>
+      </c>
+      <c r="J76" s="10" t="n">
+        <v>53.301366</v>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>PCS (INVERTER) MONTHLY AVAILABILITY (%)</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="n"/>
+      <c r="C79" s="3" t="n"/>
+      <c r="D79" s="3" t="n"/>
+      <c r="E79" s="3" t="n"/>
+      <c r="F79" s="3" t="n"/>
+      <c r="G79" s="3" t="n"/>
+      <c r="H79" s="3" t="n"/>
+      <c r="I79" s="3" t="n"/>
+      <c r="J79" s="3" t="n"/>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>PCS01</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E81" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F81" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G81" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H81" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I81" s="10" t="n">
+        <v>93.51000000000001</v>
+      </c>
+      <c r="J81" s="10" t="n">
+        <v>90.29000000000001</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>PCS02</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E82" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F82" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G82" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H82" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I82" s="10" t="n">
+        <v>93.3</v>
+      </c>
+      <c r="J82" s="10" t="n">
+        <v>86.95</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>PCS03</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E83" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F83" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G83" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H83" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I83" s="10" t="n">
+        <v>87.15000000000001</v>
+      </c>
+      <c r="J83" s="10" t="n">
+        <v>86.14</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>PCS04</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E84" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F84" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G84" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H84" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I84" s="10" t="n">
+        <v>92.36</v>
+      </c>
+      <c r="J84" s="10" t="n">
+        <v>90.29000000000001</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>PCS05</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E85" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F85" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G85" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H85" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I85" s="10" t="n">
+        <v>86.62</v>
+      </c>
+      <c r="J85" s="10" t="n">
+        <v>90.25</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>PCS06</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E86" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F86" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G86" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H86" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I86" s="10" t="n">
+        <v>93.43000000000001</v>
+      </c>
+      <c r="J86" s="10" t="n">
+        <v>90.26000000000001</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>PCS07</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E87" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F87" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G87" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H87" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I87" s="10" t="n">
+        <v>92.06999999999999</v>
+      </c>
+      <c r="J87" s="10" t="n">
+        <v>87.55</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>PCS08</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E88" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F88" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G88" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H88" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I88" s="10" t="n">
+        <v>92.64</v>
+      </c>
+      <c r="J88" s="10" t="n">
+        <v>89.79000000000001</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>PCS09</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D89" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E89" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F89" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G89" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H89" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I89" s="10" t="n">
+        <v>91.95999999999999</v>
+      </c>
+      <c r="J89" s="10" t="n">
+        <v>87.19</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>PCS10</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E90" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F90" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G90" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H90" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I90" s="10" t="n">
+        <v>93.33</v>
+      </c>
+      <c r="J90" s="10" t="n">
+        <v>90.25</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>PCS11</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E91" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F91" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G91" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H91" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I91" s="10" t="n">
+        <v>84.14</v>
+      </c>
+      <c r="J91" s="10" t="n">
+        <v>77.87</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>PCS12</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E92" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F92" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G92" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H92" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I92" s="10" t="n">
+        <v>93.19</v>
+      </c>
+      <c r="J92" s="10" t="n">
+        <v>90.25</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>PCS13</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E93" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F93" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G93" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H93" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I93" s="10" t="n">
+        <v>93.17</v>
+      </c>
+      <c r="J93" s="10" t="n">
+        <v>90.25</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>PCS14</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E94" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F94" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G94" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H94" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I94" s="10" t="n">
+        <v>93.27</v>
+      </c>
+      <c r="J94" s="10" t="n">
+        <v>87.65000000000001</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
           <t>Fleet avg</t>
         </is>
       </c>
-      <c r="B76" s="7" t="inlineStr">
+      <c r="B95" s="7" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C76" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D76" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E76" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F76" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G76" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H76" s="14" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I76" s="10" t="n">
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E95" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F95" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G95" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H95" s="14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I95" s="10" t="n">
         <v>91.43857142857144</v>
       </c>
-      <c r="J76" s="10" t="n">
+      <c r="J95" s="10" t="n">
         <v>88.21285714285715</v>
       </c>
     </row>
@@ -5569,8 +6177,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5579,8 +6187,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5589,8 +6197,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5599,8 +6207,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5609,8 +6217,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5619,8 +6227,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5629,8 +6237,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5639,8 +6247,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5649,8 +6257,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5659,8 +6267,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5669,8 +6277,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5679,8 +6287,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5689,8 +6297,8 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5699,12 +6307,12 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00059669"/>
-        <color rgb="00DC2626"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I62:J62">
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C58:J58">
     <cfRule type="colorScale" priority="45">
       <colorScale>
         <cfvo type="min"/>
@@ -5714,138 +6322,288 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I63:J63">
+  <conditionalFormatting sqref="C63:J63">
     <cfRule type="colorScale" priority="46">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I64:J64">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C64:J64">
     <cfRule type="colorScale" priority="47">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I65:J65">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C65:J65">
     <cfRule type="colorScale" priority="48">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I66:J66">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C66:J66">
     <cfRule type="colorScale" priority="49">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I67:J67">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C67:J67">
     <cfRule type="colorScale" priority="50">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I68:J68">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C68:J68">
     <cfRule type="colorScale" priority="51">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I69:J69">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C69:J69">
     <cfRule type="colorScale" priority="52">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I70:J70">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C70:J70">
     <cfRule type="colorScale" priority="53">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I71:J71">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C71:J71">
     <cfRule type="colorScale" priority="54">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I72:J72">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C72:J72">
     <cfRule type="colorScale" priority="55">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I73:J73">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C73:J73">
     <cfRule type="colorScale" priority="56">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I74:J74">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C74:J74">
     <cfRule type="colorScale" priority="57">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I75:J75">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C75:J75">
     <cfRule type="colorScale" priority="58">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="00DC2626"/>
-        <color rgb="00059669"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I76:J76">
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C76:J76">
     <cfRule type="colorScale" priority="59">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00059669"/>
+        <color rgb="00DC2626"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I81:J81">
+    <cfRule type="colorScale" priority="60">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I82:J82">
+    <cfRule type="colorScale" priority="61">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I83:J83">
+    <cfRule type="colorScale" priority="62">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I84:J84">
+    <cfRule type="colorScale" priority="63">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I85:J85">
+    <cfRule type="colorScale" priority="64">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I86:J86">
+    <cfRule type="colorScale" priority="65">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I87:J87">
+    <cfRule type="colorScale" priority="66">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I88:J88">
+    <cfRule type="colorScale" priority="67">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I89:J89">
+    <cfRule type="colorScale" priority="68">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I90:J90">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I91:J91">
+    <cfRule type="colorScale" priority="70">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I92:J92">
+    <cfRule type="colorScale" priority="71">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I93:J93">
+    <cfRule type="colorScale" priority="72">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I94:J94">
+    <cfRule type="colorScale" priority="73">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00DC2626"/>
+        <color rgb="00059669"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I95:J95">
+    <cfRule type="colorScale" priority="74">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>

</xml_diff>